<commit_message>
add function to define prepared edges input data sheet
</commit_message>
<xml_diff>
--- a/00_code_base/07_data_prep/inputs.xlsx
+++ b/00_code_base/07_data_prep/inputs.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>17.13308152456419</v>
+        <v>17133.08152456419</v>
       </c>
     </row>
     <row r="3">
@@ -496,7 +496,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>19.93655963989303</v>
+        <v>19936.55963989303</v>
       </c>
     </row>
     <row r="4">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2032.811315623034</v>
+        <v>34811.31562303352</v>
       </c>
     </row>
     <row r="5">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2029.824372234945</v>
+        <v>31824.37223494492</v>
       </c>
     </row>
     <row r="6">
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2030.796416311672</v>
+        <v>32796.41631167203</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2039.110289987785</v>
+        <v>41110.28998778499</v>
       </c>
     </row>
     <row r="8">
@@ -622,7 +622,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>21.50406118084038</v>
+        <v>21504.06118084038</v>
       </c>
     </row>
     <row r="9">
@@ -644,7 +644,7 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>10.09380869078214</v>
+        <v>10093.80869078214</v>
       </c>
     </row>
     <row r="10">
@@ -666,7 +666,7 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>13.43480786840709</v>
+        <v>13434.80786840709</v>
       </c>
     </row>
     <row r="11">
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2031.562464292669</v>
+        <v>33562.46429266888</v>
       </c>
     </row>
     <row r="12">
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2028.57552090458</v>
+        <v>30575.52090458029</v>
       </c>
     </row>
     <row r="13">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2026.428655344392</v>
+        <v>28428.65534439162</v>
       </c>
     </row>
     <row r="14">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2035.949537393924</v>
+        <v>37949.537393924</v>
       </c>
     </row>
     <row r="15">
@@ -792,7 +792,7 @@
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>17.13630021355998</v>
+        <v>17136.30021355998</v>
       </c>
     </row>
     <row r="16">
@@ -814,7 +814,7 @@
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>26.04241266489741</v>
+        <v>26042.41266489741</v>
       </c>
     </row>
     <row r="17">
@@ -836,7 +836,7 @@
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>23.43849326730724</v>
+        <v>23438.49326730724</v>
       </c>
     </row>
     <row r="18">
@@ -858,7 +858,7 @@
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>19.82712421403634</v>
+        <v>19827.12421403634</v>
       </c>
     </row>
     <row r="19">
@@ -880,7 +880,7 @@
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>20.7444505778351</v>
+        <v>20744.4505778351</v>
       </c>
     </row>
     <row r="20">
@@ -902,7 +902,7 @@
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>3.060973234991649</v>
+        <v>3060.973234991649</v>
       </c>
     </row>
     <row r="21">
@@ -924,7 +924,7 @@
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>14.07210828957255</v>
+        <v>14072.10828957254</v>
       </c>
     </row>
     <row r="22">
@@ -946,7 +946,7 @@
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>9.382478422713625</v>
+        <v>9382.478422713624</v>
       </c>
     </row>
     <row r="23">
@@ -968,7 +968,7 @@
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>26.25806482761501</v>
+        <v>26258.06482761501</v>
       </c>
     </row>
     <row r="24">
@@ -990,7 +990,7 @@
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>23.65414543002485</v>
+        <v>23654.14543002485</v>
       </c>
     </row>
     <row r="25">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>20.04277637675394</v>
+        <v>20042.77637675394</v>
       </c>
     </row>
     <row r="26">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
-        <v>20.9601027405527</v>
+        <v>20960.1027405527</v>
       </c>
     </row>
     <row r="27">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>3.276625397709252</v>
+        <v>3276.625397709252</v>
       </c>
     </row>
     <row r="28">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>14.28776045229015</v>
+        <v>14287.76045229015</v>
       </c>
     </row>
     <row r="29">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
-        <v>9.598130585431226</v>
+        <v>9598.130585431227</v>
       </c>
     </row>
     <row r="30">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>11.00791636558511</v>
+        <v>11007.91636558511</v>
       </c>
     </row>
     <row r="31">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
-        <v>33.78335969976062</v>
+        <v>33783.35969976062</v>
       </c>
     </row>
     <row r="32">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>34.69746737456359</v>
+        <v>34697.4673745636</v>
       </c>
     </row>
     <row r="33">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
-        <v>22.5823219944284</v>
+        <v>22582.3219944284</v>
       </c>
     </row>
     <row r="34">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
-        <v>28.44033596675732</v>
+        <v>28440.33596675732</v>
       </c>
     </row>
     <row r="35">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
-        <v>16.89811722787188</v>
+        <v>16898.11722787188</v>
       </c>
     </row>
     <row r="36">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
-        <v>27.6002581388574</v>
+        <v>27600.2581388574</v>
       </c>
     </row>
     <row r="37">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
-        <v>27.53266566994592</v>
+        <v>27532.66566994592</v>
       </c>
     </row>
     <row r="38">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
-        <v>10.21933756161776</v>
+        <v>10219.33756161776</v>
       </c>
     </row>
     <row r="39">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
-        <v>9.762283724216269</v>
+        <v>9762.28372421627</v>
       </c>
     </row>
     <row r="40">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
-        <v>13.4541200023818</v>
+        <v>13454.1200023818</v>
       </c>
     </row>
     <row r="41">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="n">
-        <v>8.407215656990733</v>
+        <v>8407.215656990733</v>
       </c>
     </row>
     <row r="42">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="n">
-        <v>21.42037526694997</v>
+        <v>21420.37526694997</v>
       </c>
     </row>
     <row r="43">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="n">
-        <v>25.40511224373195</v>
+        <v>25405.11224373195</v>
       </c>
     </row>
     <row r="44">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="n">
-        <v>22.92350302798162</v>
+        <v>22923.50302798162</v>
       </c>
     </row>
     <row r="45">
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>2043.906136591505</v>
+        <v>45906.13659150482</v>
       </c>
     </row>
     <row r="46">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="n">
-        <v>3.054535857000079</v>
+        <v>3054.535857000079</v>
       </c>
     </row>
     <row r="47">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>2028.630238617509</v>
+        <v>30630.23861750864</v>
       </c>
     </row>
     <row r="48">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>2038.151120667041</v>
+        <v>40151.12066704102</v>
       </c>
     </row>
     <row r="49">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="n">
-        <v>19.337883486677</v>
+        <v>19337.883486677</v>
       </c>
     </row>
     <row r="50">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="n">
-        <v>19.64365894127659</v>
+        <v>19643.65894127659</v>
       </c>
     </row>
     <row r="51">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="n">
-        <v>16.89811722787188</v>
+        <v>16898.11722787188</v>
       </c>
     </row>
     <row r="52">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="n">
-        <v>24.28822716219451</v>
+        <v>24288.22716219451</v>
       </c>
     </row>
     <row r="53">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="n">
-        <v>25.20555352599327</v>
+        <v>25205.55352599327</v>
       </c>
     </row>
     <row r="54">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="n">
-        <v>9.012329188198335</v>
+        <v>9012.329188198335</v>
       </c>
     </row>
     <row r="55">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="n">
-        <v>18.53321123773072</v>
+        <v>18533.21123773072</v>
       </c>
     </row>
     <row r="56">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="n">
-        <v>29.49284726837905</v>
+        <v>29492.84726837905</v>
       </c>
     </row>
     <row r="57">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="n">
-        <v>26.88892787078889</v>
+        <v>26888.92787078889</v>
       </c>
     </row>
     <row r="58">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="n">
-        <v>8.313873676112964</v>
+        <v>8313.873676112964</v>
       </c>
     </row>
     <row r="59">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="n">
-        <v>8.552056661801064</v>
+        <v>8552.056661801063</v>
       </c>
     </row>
     <row r="60">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="n">
-        <v>11.14631999240387</v>
+        <v>11146.31999240387</v>
       </c>
     </row>
     <row r="61">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="n">
-        <v>5.713172967518588</v>
+        <v>5713.172967518588</v>
       </c>
     </row>
     <row r="62">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="n">
-        <v>19.12545001295518</v>
+        <v>19125.45001295518</v>
       </c>
     </row>
     <row r="63">
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>2020.203710826543</v>
+        <v>22203.7108265432</v>
       </c>
     </row>
     <row r="64">
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>2014.744814289692</v>
+        <v>16744.81428969163</v>
       </c>
     </row>
     <row r="65">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>2011.80615123654</v>
+        <v>13806.15123653982</v>
       </c>
     </row>
     <row r="66">
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>2014.329603409235</v>
+        <v>16329.60340923535</v>
       </c>
     </row>
     <row r="67">
@@ -1968,7 +1968,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>2013.927267284762</v>
+        <v>15927.26728476221</v>
       </c>
     </row>
     <row r="68">
@@ -1994,7 +1994,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>2023.209966348606</v>
+        <v>25209.9663486065</v>
       </c>
     </row>
     <row r="69">
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>2020.425800367252</v>
+        <v>22425.80036725237</v>
       </c>
     </row>
     <row r="70">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>2022.595196750412</v>
+        <v>24595.19675041154</v>
       </c>
     </row>
     <row r="71">
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>2016.949616251804</v>
+        <v>18949.61625180444</v>
       </c>
     </row>
     <row r="72">
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>2014.989434653371</v>
+        <v>16989.4346533713</v>
       </c>
     </row>
     <row r="73">
@@ -2124,7 +2124,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>2011.802932547544</v>
+        <v>13802.93254754403</v>
       </c>
     </row>
     <row r="74">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>2019.605034673327</v>
+        <v>21605.03467332717</v>
       </c>
     </row>
     <row r="75">
@@ -2176,7 +2176,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>2023.892328415713</v>
+        <v>25892.32841571295</v>
       </c>
     </row>
     <row r="76">
@@ -2202,7 +2202,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>2023.892328415713</v>
+        <v>25892.32841571295</v>
       </c>
     </row>
     <row r="77">
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>2021.050226032435</v>
+        <v>23050.22603243468</v>
       </c>
     </row>
     <row r="78">
@@ -2254,7 +2254,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>2019.563191716382</v>
+        <v>21563.19171638196</v>
       </c>
     </row>
     <row r="79">
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>2023.699207075966</v>
+        <v>25699.20707596584</v>
       </c>
     </row>
     <row r="80">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="n">
-        <v>16.04838333298461</v>
+        <v>16048.38333298461</v>
       </c>
     </row>
     <row r="81">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="n">
-        <v>15.49798751470535</v>
+        <v>15497.98751470535</v>
       </c>
     </row>
     <row r="82">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="n">
-        <v>20.13289966863593</v>
+        <v>20132.89966863592</v>
       </c>
     </row>
     <row r="83">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="n">
-        <v>18.14374986924072</v>
+        <v>18143.74986924072</v>
       </c>
     </row>
     <row r="84">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="n">
-        <v>20.53523579310907</v>
+        <v>20535.23579310907</v>
       </c>
     </row>
     <row r="85">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="n">
-        <v>18.13409380225337</v>
+        <v>18134.09380225337</v>
       </c>
     </row>
     <row r="86">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="n">
-        <v>16.26081680670643</v>
+        <v>16260.81680670643</v>
       </c>
     </row>
     <row r="87">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="n">
-        <v>17.51932420405841</v>
+        <v>17519.32420405841</v>
       </c>
     </row>
     <row r="88">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="n">
-        <v>14.69331526575907</v>
+        <v>14693.31526575907</v>
       </c>
     </row>
     <row r="89">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="n">
-        <v>15.40464553382759</v>
+        <v>15404.64553382758</v>
       </c>
     </row>
     <row r="90">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="n">
-        <v>20.62857777398683</v>
+        <v>20628.57777398683</v>
       </c>
     </row>
     <row r="91">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="n">
-        <v>15.01840285433337</v>
+        <v>15018.40285433337</v>
       </c>
     </row>
     <row r="92">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="n">
-        <v>18.81645586935981</v>
+        <v>18816.45586935981</v>
       </c>
     </row>
     <row r="93">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="n">
-        <v>18.81645586935981</v>
+        <v>18816.45586935981</v>
       </c>
     </row>
     <row r="94">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="n">
-        <v>16.7854631130194</v>
+        <v>16785.4631130194</v>
       </c>
     </row>
     <row r="95">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="n">
-        <v>14.69009657676329</v>
+        <v>14690.09657676329</v>
       </c>
     </row>
     <row r="96">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="n">
-        <v>18.62333452961271</v>
+        <v>18623.3345296127</v>
       </c>
     </row>
     <row r="97">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="n">
-        <v>12.8264756482037</v>
+        <v>12826.4756482037</v>
       </c>
     </row>
     <row r="98">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="n">
-        <v>13.19984357171478</v>
+        <v>13199.84357171478</v>
       </c>
     </row>
     <row r="99">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="n">
-        <v>15.76513870135552</v>
+        <v>15765.13870135552</v>
       </c>
     </row>
     <row r="100">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="n">
-        <v>13.77598890196031</v>
+        <v>13775.98890196031</v>
       </c>
     </row>
     <row r="101">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="n">
-        <v>16.16747482582866</v>
+        <v>16167.47482582866</v>
       </c>
     </row>
     <row r="102">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="n">
-        <v>15.52373702667163</v>
+        <v>15523.73702667163</v>
       </c>
     </row>
     <row r="103">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="n">
-        <v>13.03890912192552</v>
+        <v>13038.90912192552</v>
       </c>
     </row>
     <row r="104">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="n">
-        <v>14.90896742847668</v>
+        <v>14908.96742847668</v>
       </c>
     </row>
     <row r="105">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="n">
-        <v>10.61845499709511</v>
+        <v>10618.45499709511</v>
       </c>
     </row>
     <row r="106">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="n">
-        <v>10.83410715981271</v>
+        <v>10834.10715981271</v>
       </c>
     </row>
     <row r="107">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="n">
-        <v>16.26081680670643</v>
+        <v>16260.81680670643</v>
       </c>
     </row>
     <row r="108">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="n">
-        <v>12.01536602126585</v>
+        <v>12015.36602126585</v>
       </c>
     </row>
     <row r="109">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="n">
-        <v>16.20609909377808</v>
+        <v>16206.09909377808</v>
       </c>
     </row>
     <row r="110">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="n">
-        <v>16.20609909377808</v>
+        <v>16206.09909377808</v>
       </c>
     </row>
     <row r="111">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="n">
-        <v>13.67299085409519</v>
+        <v>13672.99085409519</v>
       </c>
     </row>
     <row r="112">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="n">
-        <v>11.58406169583065</v>
+        <v>11584.06169583065</v>
       </c>
     </row>
     <row r="113">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="n">
-        <v>16.01297775403097</v>
+        <v>16012.97775403097</v>
       </c>
     </row>
     <row r="114">
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>2019.988058663826</v>
+        <v>21988.0586638256</v>
       </c>
     </row>
     <row r="115">
@@ -3080,7 +3080,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>2014.529162126974</v>
+        <v>16529.16212697403</v>
       </c>
     </row>
     <row r="116">
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>2011.590499073822</v>
+        <v>13590.49907382222</v>
       </c>
     </row>
     <row r="117">
@@ -3132,7 +3132,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>2014.113951246518</v>
+        <v>16113.95124651775</v>
       </c>
     </row>
     <row r="118">
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>2013.711615122045</v>
+        <v>15711.61512204461</v>
       </c>
     </row>
     <row r="119">
@@ -3184,7 +3184,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>2022.994314185889</v>
+        <v>24994.3141858889</v>
       </c>
     </row>
     <row r="120">
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>2020.200492137547</v>
+        <v>22200.49213754741</v>
       </c>
     </row>
     <row r="121">
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>2022.379544587694</v>
+        <v>24379.54458769394</v>
       </c>
     </row>
     <row r="122">
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>2016.733964089087</v>
+        <v>18733.96408908684</v>
       </c>
     </row>
     <row r="123">
@@ -3288,7 +3288,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>2014.773782490654</v>
+        <v>16773.7824906537</v>
       </c>
     </row>
     <row r="124">
@@ -3314,7 +3314,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>2011.587280384826</v>
+        <v>13587.28038482643</v>
       </c>
     </row>
     <row r="125">
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>2019.389382510609</v>
+        <v>21389.38251060956</v>
       </c>
     </row>
     <row r="126">
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2023.676676252995</v>
+        <v>25676.67625299534</v>
       </c>
     </row>
     <row r="127">
@@ -3392,7 +3392,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>2023.676676252995</v>
+        <v>25676.67625299534</v>
       </c>
     </row>
     <row r="128">
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>2020.834573869717</v>
+        <v>22834.57386971708</v>
       </c>
     </row>
     <row r="129">
@@ -3444,7 +3444,7 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>2019.347539553664</v>
+        <v>21347.53955366436</v>
       </c>
     </row>
     <row r="130">
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>2023.483554913248</v>
+        <v>25483.55491324823</v>
       </c>
     </row>
     <row r="131">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="n">
-        <v>13.9948597536737</v>
+        <v>13994.8597536737</v>
       </c>
     </row>
     <row r="132">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="n">
-        <v>12.96166058602668</v>
+        <v>12961.66058602668</v>
       </c>
     </row>
     <row r="133">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="n">
-        <v>15.52695571566742</v>
+        <v>15526.95571566742</v>
       </c>
     </row>
     <row r="134">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="n">
-        <v>13.53780591627221</v>
+        <v>13537.80591627221</v>
       </c>
     </row>
     <row r="135">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="n">
-        <v>15.92929184014056</v>
+        <v>15929.29184014056</v>
       </c>
     </row>
     <row r="136">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="n">
-        <v>17.001115275737</v>
+        <v>17001.115275737</v>
       </c>
     </row>
     <row r="137">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="n">
-        <v>14.20729322739552</v>
+        <v>14207.29322739552</v>
       </c>
     </row>
     <row r="138">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="n">
-        <v>16.38634567754205</v>
+        <v>16386.34567754205</v>
       </c>
     </row>
     <row r="139">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="n">
-        <v>10.90813700671577</v>
+        <v>10908.13700671577</v>
       </c>
     </row>
     <row r="140">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="n">
-        <v>10.81157633684222</v>
+        <v>10811.57633684222</v>
       </c>
     </row>
     <row r="141">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="n">
-        <v>16.02263382101833</v>
+        <v>16022.63382101833</v>
       </c>
     </row>
     <row r="142">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="n">
-        <v>13.39618360045767</v>
+        <v>13396.18360045767</v>
       </c>
     </row>
     <row r="143">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="n">
-        <v>17.68347734284345</v>
+        <v>17683.47734284345</v>
       </c>
     </row>
     <row r="144">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="E144" t="inlineStr"/>
       <c r="F144" t="n">
-        <v>17.68347734284345</v>
+        <v>17683.47734284345</v>
       </c>
     </row>
     <row r="145">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="n">
-        <v>14.84137495956519</v>
+        <v>14841.37495956519</v>
       </c>
     </row>
     <row r="146">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="n">
-        <v>13.35434064351246</v>
+        <v>13354.34064351246</v>
       </c>
     </row>
     <row r="147">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="n">
-        <v>17.49035600309634</v>
+        <v>17490.35600309634</v>
       </c>
     </row>
     <row r="148">
@@ -3870,7 +3870,7 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>2032.025955508062</v>
+        <v>34025.95550806195</v>
       </c>
     </row>
     <row r="149">
@@ -3896,7 +3896,7 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>2026.56705897121</v>
+        <v>28567.05897121038</v>
       </c>
     </row>
     <row r="150">
@@ -3922,7 +3922,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>2023.628395918058</v>
+        <v>25628.39591805857</v>
       </c>
     </row>
     <row r="151">
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>2026.151848090754</v>
+        <v>28151.8480907541</v>
       </c>
     </row>
     <row r="152">
@@ -3974,7 +3974,7 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>2025.749511966281</v>
+        <v>27749.51196628096</v>
       </c>
     </row>
     <row r="153">
@@ -4000,7 +4000,7 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>2035.032211030125</v>
+        <v>37032.21103012525</v>
       </c>
     </row>
     <row r="154">
@@ -4026,7 +4026,7 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>2032.238388981784</v>
+        <v>34238.38898178376</v>
       </c>
     </row>
     <row r="155">
@@ -4052,7 +4052,7 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>2034.41744143193</v>
+        <v>36417.44143193029</v>
       </c>
     </row>
     <row r="156">
@@ -4078,7 +4078,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>2028.771860933323</v>
+        <v>30771.86093332319</v>
       </c>
     </row>
     <row r="157">
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="F157" t="n">
-        <v>2026.81167933489</v>
+        <v>28811.67933489005</v>
       </c>
     </row>
     <row r="158">
@@ -4130,7 +4130,7 @@
         </is>
       </c>
       <c r="F158" t="n">
-        <v>2023.625177229063</v>
+        <v>25625.17722906278</v>
       </c>
     </row>
     <row r="159">
@@ -4156,7 +4156,7 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>2031.427279354846</v>
+        <v>33427.27935484592</v>
       </c>
     </row>
     <row r="160">
@@ -4182,7 +4182,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>2035.714573097232</v>
+        <v>37714.57309723169</v>
       </c>
     </row>
     <row r="161">
@@ -4208,7 +4208,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>2035.714573097232</v>
+        <v>37714.57309723169</v>
       </c>
     </row>
     <row r="162">
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>2032.872470713953</v>
+        <v>34872.47071395343</v>
       </c>
     </row>
     <row r="163">
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>2031.385436397901</v>
+        <v>33385.4363979007</v>
       </c>
     </row>
     <row r="164">
@@ -4286,7 +4286,7 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>2035.521451757485</v>
+        <v>37521.45175748458</v>
       </c>
     </row>
     <row r="165">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="E165" t="inlineStr"/>
       <c r="F165" t="n">
-        <v>10.32555429847866</v>
+        <v>10325.55429847866</v>
       </c>
     </row>
     <row r="166">
@@ -4330,7 +4330,7 @@
       </c>
       <c r="E166" t="inlineStr"/>
       <c r="F166" t="n">
-        <v>4.866657761627102</v>
+        <v>4866.657761627102</v>
       </c>
     </row>
     <row r="167">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="n">
-        <v>1.927994708475287</v>
+        <v>1927.994708475287</v>
       </c>
     </row>
     <row r="168">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="n">
-        <v>4.451446881170821</v>
+        <v>4451.446881170821</v>
       </c>
     </row>
     <row r="169">
@@ -4396,7 +4396,7 @@
       </c>
       <c r="E169" t="inlineStr"/>
       <c r="F169" t="n">
-        <v>4.04911075669768</v>
+        <v>4049.110756697681</v>
       </c>
     </row>
     <row r="170">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="n">
-        <v>13.33180982054197</v>
+        <v>13331.80982054197</v>
       </c>
     </row>
     <row r="171">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E171" t="inlineStr"/>
       <c r="F171" t="n">
-        <v>10.53798777220048</v>
+        <v>10537.98777220048</v>
       </c>
     </row>
     <row r="172">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="n">
-        <v>12.71704022234701</v>
+        <v>12717.04022234701</v>
       </c>
     </row>
     <row r="173">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="n">
-        <v>7.071459723739909</v>
+        <v>7071.459723739908</v>
       </c>
     </row>
     <row r="174">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="n">
-        <v>5.111278125306771</v>
+        <v>5111.278125306771</v>
       </c>
     </row>
     <row r="175">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="E175" t="inlineStr"/>
       <c r="F175" t="n">
-        <v>1.924776019479502</v>
+        <v>1924.776019479502</v>
       </c>
     </row>
     <row r="176">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="n">
-        <v>9.726878145262631</v>
+        <v>9726.878145262632</v>
       </c>
     </row>
     <row r="177">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="E177" t="inlineStr"/>
       <c r="F177" t="n">
-        <v>14.01417188764841</v>
+        <v>14014.17188764841</v>
       </c>
     </row>
     <row r="178">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="n">
-        <v>14.01417188764841</v>
+        <v>14014.17188764841</v>
       </c>
     </row>
     <row r="179">
@@ -4616,7 +4616,7 @@
       </c>
       <c r="E179" t="inlineStr"/>
       <c r="F179" t="n">
-        <v>11.17206950437015</v>
+        <v>11172.06950437015</v>
       </c>
     </row>
     <row r="180">
@@ -4638,7 +4638,7 @@
       </c>
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="n">
-        <v>9.685035188317427</v>
+        <v>9685.035188317426</v>
       </c>
     </row>
     <row r="181">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="n">
-        <v>13.8210505479013</v>
+        <v>13821.0505479013</v>
       </c>
     </row>
     <row r="182">
@@ -4686,7 +4686,7 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>2029.731030254067</v>
+        <v>31731.03025406715</v>
       </c>
     </row>
     <row r="183">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="F183" t="n">
-        <v>2024.272133717216</v>
+        <v>26272.13371721559</v>
       </c>
     </row>
     <row r="184">
@@ -4738,7 +4738,7 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>2021.333470664064</v>
+        <v>23333.47066406377</v>
       </c>
     </row>
     <row r="185">
@@ -4764,7 +4764,7 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>2023.856922836759</v>
+        <v>25856.92283675931</v>
       </c>
     </row>
     <row r="186">
@@ -4790,7 +4790,7 @@
         </is>
       </c>
       <c r="F186" t="n">
-        <v>2023.454586712286</v>
+        <v>25454.58671228617</v>
       </c>
     </row>
     <row r="187">
@@ -4816,7 +4816,7 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>2032.73728577613</v>
+        <v>34737.28577613045</v>
       </c>
     </row>
     <row r="188">
@@ -4842,7 +4842,7 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>2029.943463727789</v>
+        <v>31943.46372778897</v>
       </c>
     </row>
     <row r="189">
@@ -4868,7 +4868,7 @@
         </is>
       </c>
       <c r="F189" t="n">
-        <v>2032.122516177935</v>
+        <v>34122.5161779355</v>
       </c>
     </row>
     <row r="190">
@@ -4894,7 +4894,7 @@
         </is>
       </c>
       <c r="F190" t="n">
-        <v>2026.476935679328</v>
+        <v>28476.9356793284</v>
       </c>
     </row>
     <row r="191">
@@ -4920,7 +4920,7 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>2024.516754080895</v>
+        <v>26516.75408089526</v>
       </c>
     </row>
     <row r="192">
@@ -4946,7 +4946,7 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>2021.330251975068</v>
+        <v>23330.25197506799</v>
       </c>
     </row>
     <row r="193">
@@ -4972,7 +4972,7 @@
         </is>
       </c>
       <c r="F193" t="n">
-        <v>2029.132354100851</v>
+        <v>31132.35410085112</v>
       </c>
     </row>
     <row r="194">
@@ -4998,7 +4998,7 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>2033.419647843237</v>
+        <v>35419.6478432369</v>
       </c>
     </row>
     <row r="195">
@@ -5024,7 +5024,7 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>2033.419647843237</v>
+        <v>35419.6478432369</v>
       </c>
     </row>
     <row r="196">
@@ -5050,7 +5050,7 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>2030.577545459959</v>
+        <v>32577.54545995864</v>
       </c>
     </row>
     <row r="197">
@@ -5076,7 +5076,7 @@
         </is>
       </c>
       <c r="F197" t="n">
-        <v>2029.090511143906</v>
+        <v>31090.51114390591</v>
       </c>
     </row>
     <row r="198">
@@ -5102,7 +5102,7 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>2033.22652650349</v>
+        <v>35226.52650348979</v>
       </c>
     </row>
     <row r="199">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="n">
-        <v>9.150732815017095</v>
+        <v>9150.732815017096</v>
       </c>
     </row>
     <row r="200">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="n">
-        <v>9.247293484890649</v>
+        <v>9247.29348489065</v>
       </c>
     </row>
     <row r="201">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="E201" t="inlineStr"/>
       <c r="F201" t="n">
-        <v>17.96672197447254</v>
+        <v>17966.72197447254</v>
       </c>
     </row>
     <row r="202">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="E202" t="inlineStr"/>
       <c r="F202" t="n">
-        <v>15.97757217507734</v>
+        <v>15977.57217507734</v>
       </c>
     </row>
     <row r="203">
@@ -5212,7 +5212,7 @@
       </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="n">
-        <v>18.36905809894568</v>
+        <v>18369.05809894568</v>
       </c>
     </row>
     <row r="204">
@@ -5234,7 +5234,7 @@
       </c>
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="n">
-        <v>9.807345370157259</v>
+        <v>9807.34537015726</v>
       </c>
     </row>
     <row r="205">
@@ -5256,7 +5256,7 @@
       </c>
       <c r="E205" t="inlineStr"/>
       <c r="F205" t="n">
-        <v>9.099233791084535</v>
+        <v>9099.233791084534</v>
       </c>
     </row>
     <row r="206">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="E206" t="inlineStr"/>
       <c r="F206" t="n">
-        <v>9.192575771962302</v>
+        <v>9192.575771962302</v>
       </c>
     </row>
     <row r="207">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="n">
-        <v>12.35976574381486</v>
+        <v>12359.76574381486</v>
       </c>
     </row>
     <row r="208">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E208" t="inlineStr"/>
       <c r="F208" t="n">
-        <v>11.26219279625214</v>
+        <v>11262.19279625213</v>
       </c>
     </row>
     <row r="209">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="E209" t="inlineStr"/>
       <c r="F209" t="n">
-        <v>18.46240007982345</v>
+        <v>18462.40007982345</v>
       </c>
     </row>
     <row r="210">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="E210" t="inlineStr"/>
       <c r="F210" t="n">
-        <v>9.224762661920153</v>
+        <v>9224.762661920153</v>
       </c>
     </row>
     <row r="211">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="E211" t="inlineStr"/>
       <c r="F211" t="n">
-        <v>10.48970743726371</v>
+        <v>10489.70743726371</v>
       </c>
     </row>
     <row r="212">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="E212" t="inlineStr"/>
       <c r="F212" t="n">
-        <v>10.48970743726371</v>
+        <v>10489.70743726371</v>
       </c>
     </row>
     <row r="213">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="E213" t="inlineStr"/>
       <c r="F213" t="n">
-        <v>8.787020958493379</v>
+        <v>8787.020958493378</v>
       </c>
     </row>
     <row r="214">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="n">
-        <v>9.903906040030813</v>
+        <v>9903.906040030814</v>
       </c>
     </row>
     <row r="215">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="n">
-        <v>10.2965860975166</v>
+        <v>10296.5860975166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add function to update parameters of edges
relevant to, e.g., investigating if an edge fails and if the supply must be realised using other infrastructure elements.
</commit_message>
<xml_diff>
--- a/00_code_base/07_data_prep/inputs.xlsx
+++ b/00_code_base/07_data_prep/inputs.xlsx
@@ -7123,7 +7123,7 @@
         <v>61320</v>
       </c>
       <c r="F33" t="n">
-        <v>6046.273436922155</v>
+        <v>99999999</v>
       </c>
       <c r="G33" t="n">
         <v>1000000</v>
@@ -8068,7 +8068,7 @@
         <v>513190</v>
       </c>
       <c r="F60" t="n">
-        <v>7933.699335456246</v>
+        <v>99999999</v>
       </c>
       <c r="G60" t="n">
         <v>1000000</v>
@@ -8488,7 +8488,7 @@
         <v>486910</v>
       </c>
       <c r="F72" t="n">
-        <v>6680.697912429536</v>
+        <v>99999999</v>
       </c>
       <c r="G72" t="n">
         <v>1000000</v>
@@ -8663,7 +8663,7 @@
         <v>439277.4999999999</v>
       </c>
       <c r="F77" t="n">
-        <v>6280.109140649178</v>
+        <v>99999999</v>
       </c>
       <c r="G77" t="n">
         <v>1000000</v>
@@ -9153,7 +9153,7 @@
         <v>80300</v>
       </c>
       <c r="F91" t="n">
-        <v>5049.665540931014</v>
+        <v>99999999</v>
       </c>
       <c r="G91" t="n">
         <v>1000000</v>
@@ -9468,7 +9468,7 @@
         <v>349998.5</v>
       </c>
       <c r="F100" t="n">
-        <v>7960.512506379757</v>
+        <v>99999999</v>
       </c>
       <c r="G100" t="n">
         <v>1000000</v>

</xml_diff>

<commit_message>
model testing with import and export nodes for LNG
</commit_message>
<xml_diff>
--- a/00_code_base/07_data_prep/inputs.xlsx
+++ b/00_code_base/07_data_prep/inputs.xlsx
@@ -32220,7 +32220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C337"/>
+  <dimension ref="A1:C449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33928,7 +33928,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>AL_LNG</t>
+          <t>AL_LNG_exp</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -33943,7 +33943,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>AT_LNG</t>
+          <t>AT_LNG_exp</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -33958,7 +33958,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>BE_LNG</t>
+          <t>BE_LNG_exp</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -33973,7 +33973,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>BA_LNG</t>
+          <t>BA_LNG_exp</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -33988,7 +33988,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>BG_LNG</t>
+          <t>BG_LNG_exp</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -34003,7 +34003,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>HR_LNG</t>
+          <t>HR_LNG_exp</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -34018,7 +34018,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>CZ_LNG</t>
+          <t>CZ_LNG_exp</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -34033,7 +34033,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>DK_LNG</t>
+          <t>DK_LNG_exp</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -34048,7 +34048,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>EE_LNG</t>
+          <t>EE_LNG_exp</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -34063,7 +34063,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>FI_LNG</t>
+          <t>FI_LNG_exp</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -34078,7 +34078,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>FR_LNG</t>
+          <t>FR_LNG_exp</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -34093,7 +34093,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>DE_LNG</t>
+          <t>DE_LNG_exp</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -34108,7 +34108,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>EL_LNG</t>
+          <t>EL_LNG_exp</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -34123,7 +34123,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>HU_LNG</t>
+          <t>HU_LNG_exp</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -34138,7 +34138,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>IE_LNG</t>
+          <t>IE_LNG_exp</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -34153,7 +34153,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>IT_LNG</t>
+          <t>IT_LNG_exp</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -34168,7 +34168,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>LV_LNG</t>
+          <t>LV_LNG_exp</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -34183,7 +34183,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>LT_LNG</t>
+          <t>LT_LNG_exp</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -34198,7 +34198,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LU_LNG</t>
+          <t>LU_LNG_exp</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -34213,7 +34213,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>MD_LNG</t>
+          <t>MD_LNG_exp</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -34228,7 +34228,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>NL_LNG</t>
+          <t>NL_LNG_exp</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -34243,7 +34243,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>MK_LNG</t>
+          <t>MK_LNG_exp</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -34258,7 +34258,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>NO_LNG</t>
+          <t>NO_LNG_exp</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -34273,7 +34273,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>PL_LNG</t>
+          <t>PL_LNG_exp</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -34288,7 +34288,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>PT_LNG</t>
+          <t>PT_LNG_exp</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -34303,7 +34303,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>RO_LNG</t>
+          <t>RO_LNG_exp</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -34318,7 +34318,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>RS_LNG</t>
+          <t>RS_LNG_exp</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -34333,7 +34333,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>SK_LNG</t>
+          <t>SK_LNG_exp</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -34348,7 +34348,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>SI_LNG</t>
+          <t>SI_LNG_exp</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -34363,7 +34363,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>ES_LNG</t>
+          <t>ES_LNG_exp</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -34378,7 +34378,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>SE_LNG</t>
+          <t>SE_LNG_exp</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -34393,7 +34393,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>CH_LNG</t>
+          <t>CH_LNG_exp</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -34408,7 +34408,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>TR_LNG</t>
+          <t>TR_LNG_exp</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -34423,7 +34423,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>UK_LNG</t>
+          <t>UK_LNG_exp</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -34438,7 +34438,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>UA_LNG</t>
+          <t>UA_LNG_exp</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -34453,7 +34453,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>USA_LNG</t>
+          <t>USA_LNG_exp</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -34468,7 +34468,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>CM_LNG</t>
+          <t>CM_LNG_exp</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -34483,7 +34483,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>SA_LNG</t>
+          <t>SA_LNG_exp</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -34498,7 +34498,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>TT_LNG</t>
+          <t>TT_LNG_exp</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -34513,7 +34513,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>ME_LNG</t>
+          <t>ME_LNG_exp</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -34528,7 +34528,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>QA_LNG</t>
+          <t>QA_LNG_exp</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -34543,7 +34543,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>AF_LNG</t>
+          <t>AF_LNG_exp</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -34558,7 +34558,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>AU_LNG</t>
+          <t>AU_LNG_exp</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -34573,7 +34573,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>CN_LNG</t>
+          <t>CN_LNG_exp</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -34588,7 +34588,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>JS_LNG</t>
+          <t>JS_LNG_exp</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -34603,7 +34603,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>IN_LNG</t>
+          <t>IN_LNG_exp</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -34618,7 +34618,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>AS_LNG</t>
+          <t>AS_LNG_exp</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -34633,7 +34633,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CR_LNG</t>
+          <t>CR_LNG_exp</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -34648,7 +34648,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>RU_LNG</t>
+          <t>RU_LNG_exp</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -34663,7 +34663,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>DZ_LNG</t>
+          <t>DZ_LNG_exp</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -34678,7 +34678,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>LY_LNG</t>
+          <t>LY_LNG_exp</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -34693,7 +34693,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>TN_LNG</t>
+          <t>TN_LNG_exp</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -34708,7 +34708,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>MA_LNG</t>
+          <t>MA_LNG_exp</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -34723,7 +34723,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>EG_LNG</t>
+          <t>EG_LNG_exp</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -34738,7 +34738,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>IM_LNG</t>
+          <t>IM_LNG_exp</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -34753,7 +34753,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>BY_LNG</t>
+          <t>BY_LNG_exp</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -34763,12 +34763,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AL_LNG_imp</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -34778,12 +34778,12 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>AT_LNG_imp</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -34793,12 +34793,12 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BE_LNG_imp</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -34808,12 +34808,12 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>BA_LNG_imp</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -34823,12 +34823,12 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>BG</t>
+          <t>BG_LNG_imp</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -34838,12 +34838,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>HR_LNG_imp</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -34853,12 +34853,12 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>CZ_LNG_imp</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -34868,12 +34868,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>DK_LNG_imp</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -34883,12 +34883,12 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>EE</t>
+          <t>EE_LNG_imp</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -34898,12 +34898,12 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>FI_LNG_imp</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -34913,12 +34913,12 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>FR_LNG_imp</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -34928,12 +34928,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>DE_LNG_imp</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -34943,12 +34943,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>EL_LNG_imp</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -34958,12 +34958,12 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>HU</t>
+          <t>HU_LNG_imp</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -34973,12 +34973,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>IE_LNG_imp</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -34988,12 +34988,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>IT_LNG_imp</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -35003,12 +35003,12 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>LV_LNG_imp</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -35018,12 +35018,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>LT_LNG_imp</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -35033,12 +35033,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>LU_LNG_imp</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -35048,12 +35048,12 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>MD_LNG_imp</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -35063,12 +35063,12 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>NL_LNG_imp</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -35078,12 +35078,12 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>MK</t>
+          <t>MK_LNG_imp</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -35093,12 +35093,12 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>NO_LNG_imp</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -35108,12 +35108,12 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PL_LNG_imp</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -35123,12 +35123,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>PT_LNG_imp</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -35138,12 +35138,12 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RO_LNG_imp</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -35153,12 +35153,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RS_LNG_imp</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -35168,12 +35168,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>SK_LNG_imp</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -35183,12 +35183,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SI_LNG_imp</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -35198,12 +35198,12 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>ES_LNG_imp</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -35213,12 +35213,12 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SE_LNG_imp</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -35228,12 +35228,12 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>CH_LNG_imp</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -35243,12 +35243,12 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>TR_LNG_imp</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -35258,12 +35258,12 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>UK_LNG_imp</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -35273,12 +35273,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>UA</t>
+          <t>UA_LNG_imp</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -35288,12 +35288,12 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>AL_Prod</t>
+          <t>USA_LNG_imp</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -35303,12 +35303,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>DZ_Prod</t>
+          <t>CM_LNG_imp</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -35318,12 +35318,12 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>AT_Prod</t>
+          <t>SA_LNG_imp</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -35333,12 +35333,12 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>BY_Prod</t>
+          <t>TT_LNG_imp</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -35348,12 +35348,12 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>BE_Prod</t>
+          <t>ME_LNG_imp</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -35363,12 +35363,12 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>BA_Prod</t>
+          <t>QA_LNG_imp</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -35378,12 +35378,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>BG_Prod</t>
+          <t>AF_LNG_imp</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -35393,12 +35393,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>HR_Prod</t>
+          <t>AU_LNG_imp</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -35408,12 +35408,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>CZ_Prod</t>
+          <t>CN_LNG_imp</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -35423,12 +35423,12 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>DK_Prod</t>
+          <t>JS_LNG_imp</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -35438,12 +35438,12 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>EE_Prod</t>
+          <t>IN_LNG_imp</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -35453,12 +35453,12 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>FI_Prod</t>
+          <t>AS_LNG_imp</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -35468,12 +35468,12 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>FR_Prod</t>
+          <t>CR_LNG_imp</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -35483,12 +35483,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>DE_Prod</t>
+          <t>RU_LNG_imp</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -35498,12 +35498,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>EL_Prod</t>
+          <t>DZ_LNG_imp</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -35513,12 +35513,12 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>HU_Prod</t>
+          <t>LY_LNG_imp</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -35528,12 +35528,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>IE_Prod</t>
+          <t>TN_LNG_imp</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -35543,12 +35543,12 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>IT_Prod</t>
+          <t>MA_LNG_imp</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -35558,12 +35558,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>LV_Prod</t>
+          <t>EG_LNG_imp</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -35573,12 +35573,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>LY_Prod</t>
+          <t>IM_LNG_imp</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -35588,12 +35588,12 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Methane</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>LT_Prod</t>
+          <t>BY_LNG_imp</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -35608,7 +35608,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>LU_Prod</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -35623,7 +35623,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>MD_Prod</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -35638,7 +35638,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>NL_Prod</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -35653,7 +35653,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>MK_Prod</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -35668,7 +35668,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>NO_Prod</t>
+          <t>BG</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -35683,7 +35683,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>PL_Prod</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -35698,7 +35698,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>PT_Prod</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -35713,7 +35713,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>RO_Prod</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -35728,7 +35728,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>RU_Prod</t>
+          <t>EE</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -35743,7 +35743,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>RS_Prod</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -35758,7 +35758,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>SK_Prod</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -35773,7 +35773,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>SI_Prod</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -35788,7 +35788,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>CH_Prod</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -35803,7 +35803,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>TN_Prod</t>
+          <t>HU</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -35818,7 +35818,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>TR_Prod</t>
+          <t>IE</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -35833,7 +35833,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>UK_Prod</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -35848,7 +35848,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>UA_Prod</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -35863,7 +35863,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>ES_Prod</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -35878,7 +35878,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>LU</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -35893,7 +35893,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>CM</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -35908,7 +35908,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -35923,7 +35923,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>MK</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -35938,7 +35938,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -35953,7 +35953,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -35968,7 +35968,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>AF</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -35983,7 +35983,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -35998,7 +35998,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -36013,7 +36013,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>JS</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -36028,7 +36028,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -36043,7 +36043,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>AS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -36058,7 +36058,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -36073,7 +36073,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -36088,7 +36088,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>DZ</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -36103,7 +36103,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>LY</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -36118,7 +36118,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>UA</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -36133,7 +36133,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>AL_Prod</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -36148,7 +36148,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>DZ_Prod</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -36163,7 +36163,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>IM</t>
+          <t>AT_Prod</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -36178,7 +36178,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>BY</t>
+          <t>BY_Prod</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -36193,7 +36193,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>USA_Prod</t>
+          <t>BE_Prod</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -36208,7 +36208,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>CM_Prod</t>
+          <t>BA_Prod</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -36223,7 +36223,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>SA_Prod</t>
+          <t>BG_Prod</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -36238,7 +36238,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>TT_Prod</t>
+          <t>HR_Prod</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -36253,7 +36253,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>ME_Prod</t>
+          <t>CZ_Prod</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -36268,7 +36268,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>QA_Prod</t>
+          <t>DK_Prod</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -36283,7 +36283,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>AF_Prod</t>
+          <t>EE_Prod</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -36298,7 +36298,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>MA_Prod</t>
+          <t>FI_Prod</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -36313,7 +36313,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>AU_Prod</t>
+          <t>FR_Prod</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -36328,7 +36328,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>CN_Prod</t>
+          <t>DE_Prod</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -36343,7 +36343,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>JS_Prod</t>
+          <t>EL_Prod</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -36358,7 +36358,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>IN_Prod</t>
+          <t>HU_Prod</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -36373,7 +36373,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>AS_Prod</t>
+          <t>IE_Prod</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -36388,7 +36388,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>CR_Prod</t>
+          <t>IT_Prod</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -36403,7 +36403,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>EG_Prod</t>
+          <t>LV_Prod</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -36418,7 +36418,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>IM_Prod</t>
+          <t>LY_Prod</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -36433,7 +36433,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>SE_Prod</t>
+          <t>LT_Prod</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -36448,7 +36448,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>AL_LNG</t>
+          <t>LU_Prod</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -36463,7 +36463,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>AT_LNG</t>
+          <t>MD_Prod</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -36478,7 +36478,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>BE_LNG</t>
+          <t>NL_Prod</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -36493,7 +36493,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>BA_LNG</t>
+          <t>MK_Prod</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -36508,7 +36508,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>BG_LNG</t>
+          <t>NO_Prod</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -36523,7 +36523,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>HR_LNG</t>
+          <t>PL_Prod</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -36538,7 +36538,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>CZ_LNG</t>
+          <t>PT_Prod</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -36553,7 +36553,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>DK_LNG</t>
+          <t>RO_Prod</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -36568,7 +36568,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>EE_LNG</t>
+          <t>RU_Prod</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -36583,7 +36583,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>FI_LNG</t>
+          <t>RS_Prod</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -36598,7 +36598,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>FR_LNG</t>
+          <t>SK_Prod</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -36613,7 +36613,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>DE_LNG</t>
+          <t>SI_Prod</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -36628,7 +36628,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>EL_LNG</t>
+          <t>CH_Prod</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -36643,7 +36643,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>HU_LNG</t>
+          <t>TN_Prod</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -36658,7 +36658,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>IE_LNG</t>
+          <t>TR_Prod</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -36673,7 +36673,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>IT_LNG</t>
+          <t>UK_Prod</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -36688,7 +36688,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>LV_LNG</t>
+          <t>UA_Prod</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -36703,7 +36703,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>LT_LNG</t>
+          <t>ES_Prod</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -36718,7 +36718,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>LU_LNG</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -36733,7 +36733,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>MD_LNG</t>
+          <t>CM</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -36748,7 +36748,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>NL_LNG</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -36763,7 +36763,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>MK_LNG</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -36778,7 +36778,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>NO_LNG</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -36793,7 +36793,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>PL_LNG</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -36808,7 +36808,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>PT_LNG</t>
+          <t>AF</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -36823,7 +36823,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>RO_LNG</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -36838,7 +36838,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>RS_LNG</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36853,7 +36853,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>SK_LNG</t>
+          <t>JS</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36868,7 +36868,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>SI_LNG</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36883,7 +36883,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>ES_LNG</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36898,7 +36898,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>SE_LNG</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36913,7 +36913,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>CH_LNG</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36928,7 +36928,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>TR_LNG</t>
+          <t>DZ</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36943,7 +36943,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>UK_LNG</t>
+          <t>LY</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36958,7 +36958,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>UA_LNG</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36973,7 +36973,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>USA_LNG</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36988,7 +36988,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>CM_LNG</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37003,7 +37003,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>SA_LNG</t>
+          <t>IM</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37018,7 +37018,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>TT_LNG</t>
+          <t>BY</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37033,7 +37033,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>ME_LNG</t>
+          <t>USA_Prod</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37048,7 +37048,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>QA_LNG</t>
+          <t>CM_Prod</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37063,7 +37063,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>AF_LNG</t>
+          <t>SA_Prod</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37078,7 +37078,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>AU_LNG</t>
+          <t>TT_Prod</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37093,7 +37093,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>CN_LNG</t>
+          <t>ME_Prod</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37108,7 +37108,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>JS_LNG</t>
+          <t>QA_Prod</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37123,7 +37123,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>IN_LNG</t>
+          <t>AF_Prod</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37138,7 +37138,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>AS_LNG</t>
+          <t>MA_Prod</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37153,7 +37153,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>CR_LNG</t>
+          <t>AU_Prod</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -37168,7 +37168,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>RU_LNG</t>
+          <t>CN_Prod</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -37183,7 +37183,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>DZ_LNG</t>
+          <t>JS_Prod</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -37198,7 +37198,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>LY_LNG</t>
+          <t>IN_Prod</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -37213,7 +37213,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>TN_LNG</t>
+          <t>AS_Prod</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -37228,7 +37228,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>MA_LNG</t>
+          <t>CR_Prod</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -37243,7 +37243,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>EG_LNG</t>
+          <t>EG_Prod</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -37258,7 +37258,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>IM_LNG</t>
+          <t>IM_Prod</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -37273,10 +37273,1690 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>BY_LNG</t>
+          <t>SE_Prod</t>
         </is>
       </c>
       <c r="C337" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>AL_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>AT_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>BE_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>BA_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>BG_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C342" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>HR_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C343" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>CZ_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C344" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>DK_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C345" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>EE_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C346" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>FI_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C347" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>FR_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C348" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>DE_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C349" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>EL_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C350" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>HU_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C351" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>IE_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C352" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>IT_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C353" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>LV_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C354" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>LT_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>LU_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C356" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>MD_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>NL_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>MK_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>NO_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>PL_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>PT_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>RO_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>RS_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>SK_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>SI_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>ES_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>SE_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>CH_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>TR_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>UK_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>UA_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>USA_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>CM_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>SA_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>TT_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>ME_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>QA_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>AF_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>AU_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>CN_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>JS_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>IN_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>AS_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>CR_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>RU_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>DZ_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>LY_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C388" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>TN_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C389" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>MA_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C390" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>EG_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C391" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>IM_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C392" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>BY_LNG_exp</t>
+        </is>
+      </c>
+      <c r="C393" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>AL_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C394" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>AT_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>BE_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>BA_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>BG_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>HR_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C399" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>CZ_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>DK_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>EE_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>FI_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C403" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>FR_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C404" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>DE_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>EL_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>HU_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>IE_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>IT_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>LV_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>LT_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C411" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>LU_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>MD_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>NL_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>MK_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>NO_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>PL_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>PT_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>RO_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>RS_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>SK_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>SI_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C422" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>ES_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>SE_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>CH_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>TR_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>UK_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C427" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>UA_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C428" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>USA_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C429" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>CM_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C430" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>SA_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C431" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>TT_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C432" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>ME_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C433" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>QA_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C434" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>AF_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C435" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>AU_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C436" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>CN_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C437" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>JS_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C438" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>IN_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C439" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>AS_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C440" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>CR_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C441" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>RU_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C442" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>DZ_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C443" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>LY_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C444" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>TN_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C445" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>MA_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C446" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>EG_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C447" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>IM_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C448" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>BY_LNG_imp</t>
+        </is>
+      </c>
+      <c r="C449" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>